<commit_message>
Add Payable Due Date Terms; EOD graph, reports, dashboard, and UX improvements
Payables:
- Add PayableTerms table (PayableTerm model, PayableTermService, PayableTerms admin page)
- Due Date Term dropdown on vendor invoice with calculated due date label
- DueDateTermID FK added to PayableHeaders; Portal_Full.sql updated with table, column, and 10 seed terms
- DueDateTerms_Import_Template.xlsx added to SampleData

EOD Sales / Dashboard / Reports:
- EOD graph (LineGraph.razor shared component, portal.js, EodSections graph toggle)
- Dashboard service and updated Home page
- Reports module (Reports.razor, ReportViewer.razor, ReportService, ReportDef model)
- EodSalesService, EodSectionService, EodRowService, EodSetupService enhancements

General:
- ChartOfAccounts page and service improvements
- App.razor, NavMenu updates
- app.css and portal.js additions
- SampleData file renames and updates

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SampleData/Vendors.xlsx
+++ b/SampleData/Vendors.xlsx
@@ -36,7 +36,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -45,7 +45,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="004472C4"/>
+        <fgColor rgb="002B6B35"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F0F7F0"/>
       </patternFill>
     </fill>
   </fills>
@@ -61,12 +66,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -448,7 +458,7 @@
     <col width="26" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="20" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>VendorCode</t>
@@ -550,56 +560,56 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>001-2100</t>
+          <t>01-000-2000</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>USFDS01</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>US Foods</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>National broadline distributor</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>9399 W Higgins Rd</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr"/>
-      <c r="F3" s="2" t="inlineStr"/>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr"/>
+      <c r="F3" s="3" t="inlineStr"/>
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>Rosemont</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>IL</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>60018</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>001-2100</t>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>01-000-2000</t>
         </is>
       </c>
     </row>
@@ -648,56 +658,56 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>001-2100</t>
+          <t>01-000-2000</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>GPFSC01</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Gordon Food Service</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>Broadline food distributor</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>1300 Gezon Pkwy SW</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="2" t="inlineStr"/>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr"/>
+      <c r="F5" s="3" t="inlineStr"/>
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>Wyoming</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>MI</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>49509</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>001-2100</t>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>01-000-2000</t>
         </is>
       </c>
     </row>
@@ -746,56 +756,56 @@
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>001-2100</t>
+          <t>01-000-2000</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>BENCO01</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Ben E Keith Foods</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>Southwest food distributor</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>601 E 7th St</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr"/>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr"/>
+      <c r="F7" s="3" t="inlineStr"/>
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>Fort Worth</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H7" s="3" t="inlineStr">
         <is>
           <t>TX</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="I7" s="3" t="inlineStr">
         <is>
           <t>76102</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="K7" s="2" t="inlineStr">
-        <is>
-          <t>001-2100</t>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t>01-000-2000</t>
         </is>
       </c>
     </row>
@@ -844,56 +854,56 @@
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>001-2100</t>
+          <t>01-000-2000</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>TAYFM01</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>Taylor Farms</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>Fresh-cut produce and salads</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>10 Becerra Rd</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr"/>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="E9" s="3" t="inlineStr"/>
+      <c r="F9" s="3" t="inlineStr"/>
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>Salinas</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H9" s="3" t="inlineStr">
         <is>
           <t>CA</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="I9" s="3" t="inlineStr">
         <is>
           <t>93905</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="K9" s="2" t="inlineStr">
-        <is>
-          <t>001-2100</t>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>01-000-2000</t>
         </is>
       </c>
     </row>
@@ -942,56 +952,56 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>001-2100</t>
+          <t>01-000-2000</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>TYSON01</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>Tyson Foods</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>Poultry and protein distributor</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D11" s="3" t="inlineStr">
         <is>
           <t>2200 Don Tyson Pkwy</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr"/>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="E11" s="3" t="inlineStr"/>
+      <c r="F11" s="3" t="inlineStr"/>
+      <c r="G11" s="3" t="inlineStr">
         <is>
           <t>Springdale</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H11" s="3" t="inlineStr">
         <is>
           <t>AR</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="I11" s="3" t="inlineStr">
         <is>
           <t>72762</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="K11" s="2" t="inlineStr">
-        <is>
-          <t>001-2100</t>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t>01-000-2000</t>
         </is>
       </c>
     </row>
@@ -1040,56 +1050,56 @@
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>001-2100</t>
+          <t>01-000-2000</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>LANDB01</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>Land O Lakes</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>Dairy products supplier</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D13" s="3" t="inlineStr">
         <is>
           <t>4001 Lexington Ave N</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr"/>
-      <c r="F13" s="2" t="inlineStr"/>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="E13" s="3" t="inlineStr"/>
+      <c r="F13" s="3" t="inlineStr"/>
+      <c r="G13" s="3" t="inlineStr">
         <is>
           <t>Arden Hills</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="H13" s="3" t="inlineStr">
         <is>
           <t>MN</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="I13" s="3" t="inlineStr">
         <is>
           <t>55126</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="K13" s="2" t="inlineStr">
-        <is>
-          <t>001-2100</t>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>01-000-2000</t>
         </is>
       </c>
     </row>
@@ -1138,56 +1148,56 @@
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>001-2100</t>
+          <t>01-000-2000</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>KEHNE01</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>Kehe Distributors</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
         <is>
           <t>Natural and specialty grocery</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="D15" s="3" t="inlineStr">
         <is>
           <t>900 S Milwaukee Ave</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr"/>
-      <c r="F15" s="2" t="inlineStr"/>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="E15" s="3" t="inlineStr"/>
+      <c r="F15" s="3" t="inlineStr"/>
+      <c r="G15" s="3" t="inlineStr">
         <is>
           <t>Wheeling</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr">
+      <c r="H15" s="3" t="inlineStr">
         <is>
           <t>IL</t>
         </is>
       </c>
-      <c r="I15" s="2" t="inlineStr">
+      <c r="I15" s="3" t="inlineStr">
         <is>
           <t>60090</t>
         </is>
       </c>
-      <c r="J15" s="2" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="K15" s="2" t="inlineStr">
-        <is>
-          <t>001-2100</t>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="K15" s="3" t="inlineStr">
+        <is>
+          <t>01-000-2000</t>
         </is>
       </c>
     </row>
@@ -1240,56 +1250,56 @@
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>001-2100</t>
+          <t>01-000-2000</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>OTTFD01</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>Otis Spunkmeyer</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr">
         <is>
           <t>Bakery and dessert products</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="D17" s="3" t="inlineStr">
         <is>
           <t>7090 Mowry Ave</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr"/>
-      <c r="F17" s="2" t="inlineStr"/>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="E17" s="3" t="inlineStr"/>
+      <c r="F17" s="3" t="inlineStr"/>
+      <c r="G17" s="3" t="inlineStr">
         <is>
           <t>Newark</t>
         </is>
       </c>
-      <c r="H17" s="2" t="inlineStr">
+      <c r="H17" s="3" t="inlineStr">
         <is>
           <t>CA</t>
         </is>
       </c>
-      <c r="I17" s="2" t="inlineStr">
+      <c r="I17" s="3" t="inlineStr">
         <is>
           <t>94560</t>
         </is>
       </c>
-      <c r="J17" s="2" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="K17" s="2" t="inlineStr">
-        <is>
-          <t>001-2100</t>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="K17" s="3" t="inlineStr">
+        <is>
+          <t>01-000-2000</t>
         </is>
       </c>
     </row>
@@ -1338,60 +1348,60 @@
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>002-2100</t>
+          <t>01-000-2000</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>GLAZR01</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>Glazers Distributors</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="C19" s="3" t="inlineStr">
         <is>
           <t>Beer wine and spirits</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="D19" s="3" t="inlineStr">
         <is>
           <t>14911 Quorum Dr</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="E19" s="3" t="inlineStr">
         <is>
           <t>Ste 300</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr"/>
-      <c r="G19" s="2" t="inlineStr">
+      <c r="F19" s="3" t="inlineStr"/>
+      <c r="G19" s="3" t="inlineStr">
         <is>
           <t>Dallas</t>
         </is>
       </c>
-      <c r="H19" s="2" t="inlineStr">
+      <c r="H19" s="3" t="inlineStr">
         <is>
           <t>TX</t>
         </is>
       </c>
-      <c r="I19" s="2" t="inlineStr">
+      <c r="I19" s="3" t="inlineStr">
         <is>
           <t>75254</t>
         </is>
       </c>
-      <c r="J19" s="2" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="K19" s="2" t="inlineStr">
-        <is>
-          <t>002-2100</t>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="K19" s="3" t="inlineStr">
+        <is>
+          <t>01-000-2000</t>
         </is>
       </c>
     </row>
@@ -1440,56 +1450,56 @@
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>002-2100</t>
+          <t>01-000-2000</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>REYES01</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>Reyes Beer Division</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C21" s="3" t="inlineStr">
         <is>
           <t>Beer and malt beverage distributor</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="D21" s="3" t="inlineStr">
         <is>
           <t>6250 N River Rd</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr"/>
-      <c r="F21" s="2" t="inlineStr"/>
-      <c r="G21" s="2" t="inlineStr">
+      <c r="E21" s="3" t="inlineStr"/>
+      <c r="F21" s="3" t="inlineStr"/>
+      <c r="G21" s="3" t="inlineStr">
         <is>
           <t>Rosemont</t>
         </is>
       </c>
-      <c r="H21" s="2" t="inlineStr">
+      <c r="H21" s="3" t="inlineStr">
         <is>
           <t>IL</t>
         </is>
       </c>
-      <c r="I21" s="2" t="inlineStr">
+      <c r="I21" s="3" t="inlineStr">
         <is>
           <t>60018</t>
         </is>
       </c>
-      <c r="J21" s="2" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="K21" s="2" t="inlineStr">
-        <is>
-          <t>002-2100</t>
+      <c r="J21" s="3" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="K21" s="3" t="inlineStr">
+        <is>
+          <t>01-000-2000</t>
         </is>
       </c>
     </row>
@@ -1538,56 +1548,56 @@
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>001-2100</t>
+          <t>01-000-2000</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>PEPSI01</t>
         </is>
       </c>
-      <c r="B23" s="2" t="inlineStr">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>PepsiCo Foodservice</t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr">
+      <c r="C23" s="3" t="inlineStr">
         <is>
           <t>Beverages and snack foods</t>
         </is>
       </c>
-      <c r="D23" s="2" t="inlineStr">
+      <c r="D23" s="3" t="inlineStr">
         <is>
           <t>700 Anderson Hill Rd</t>
         </is>
       </c>
-      <c r="E23" s="2" t="inlineStr"/>
-      <c r="F23" s="2" t="inlineStr"/>
-      <c r="G23" s="2" t="inlineStr">
+      <c r="E23" s="3" t="inlineStr"/>
+      <c r="F23" s="3" t="inlineStr"/>
+      <c r="G23" s="3" t="inlineStr">
         <is>
           <t>Purchase</t>
         </is>
       </c>
-      <c r="H23" s="2" t="inlineStr">
+      <c r="H23" s="3" t="inlineStr">
         <is>
           <t>NY</t>
         </is>
       </c>
-      <c r="I23" s="2" t="inlineStr">
+      <c r="I23" s="3" t="inlineStr">
         <is>
           <t>10577</t>
         </is>
       </c>
-      <c r="J23" s="2" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="K23" s="2" t="inlineStr">
-        <is>
-          <t>001-2100</t>
+      <c r="J23" s="3" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="K23" s="3" t="inlineStr">
+        <is>
+          <t>01-000-2000</t>
         </is>
       </c>
     </row>
@@ -1636,56 +1646,56 @@
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>001-2100</t>
+          <t>01-000-2000</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>CINTA01</t>
         </is>
       </c>
-      <c r="B25" s="2" t="inlineStr">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>Cintas Corporation</t>
         </is>
       </c>
-      <c r="C25" s="2" t="inlineStr">
+      <c r="C25" s="3" t="inlineStr">
         <is>
           <t>Uniforms and linen services</t>
         </is>
       </c>
-      <c r="D25" s="2" t="inlineStr">
+      <c r="D25" s="3" t="inlineStr">
         <is>
           <t>6800 Cintas Blvd</t>
         </is>
       </c>
-      <c r="E25" s="2" t="inlineStr"/>
-      <c r="F25" s="2" t="inlineStr"/>
-      <c r="G25" s="2" t="inlineStr">
+      <c r="E25" s="3" t="inlineStr"/>
+      <c r="F25" s="3" t="inlineStr"/>
+      <c r="G25" s="3" t="inlineStr">
         <is>
           <t>Mason</t>
         </is>
       </c>
-      <c r="H25" s="2" t="inlineStr">
+      <c r="H25" s="3" t="inlineStr">
         <is>
           <t>OH</t>
         </is>
       </c>
-      <c r="I25" s="2" t="inlineStr">
+      <c r="I25" s="3" t="inlineStr">
         <is>
           <t>45040</t>
         </is>
       </c>
-      <c r="J25" s="2" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="K25" s="2" t="inlineStr">
-        <is>
-          <t>001-2100</t>
+      <c r="J25" s="3" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="K25" s="3" t="inlineStr">
+        <is>
+          <t>01-000-2000</t>
         </is>
       </c>
     </row>
@@ -1734,56 +1744,56 @@
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>001-2100</t>
+          <t>01-000-2000</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>NTRST01</t>
         </is>
       </c>
-      <c r="B27" s="2" t="inlineStr">
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>National Restaurant Supply</t>
         </is>
       </c>
-      <c r="C27" s="2" t="inlineStr">
+      <c r="C27" s="3" t="inlineStr">
         <is>
           <t>Commercial kitchen equipment</t>
         </is>
       </c>
-      <c r="D27" s="2" t="inlineStr">
+      <c r="D27" s="3" t="inlineStr">
         <is>
           <t>3850 Forest Ln</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr"/>
-      <c r="F27" s="2" t="inlineStr"/>
-      <c r="G27" s="2" t="inlineStr">
+      <c r="E27" s="3" t="inlineStr"/>
+      <c r="F27" s="3" t="inlineStr"/>
+      <c r="G27" s="3" t="inlineStr">
         <is>
           <t>Dallas</t>
         </is>
       </c>
-      <c r="H27" s="2" t="inlineStr">
+      <c r="H27" s="3" t="inlineStr">
         <is>
           <t>TX</t>
         </is>
       </c>
-      <c r="I27" s="2" t="inlineStr">
+      <c r="I27" s="3" t="inlineStr">
         <is>
           <t>75234</t>
         </is>
       </c>
-      <c r="J27" s="2" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="K27" s="2" t="inlineStr">
-        <is>
-          <t>001-2100</t>
+      <c r="J27" s="3" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="K27" s="3" t="inlineStr">
+        <is>
+          <t>01-000-2000</t>
         </is>
       </c>
     </row>
@@ -1832,56 +1842,56 @@
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>001-2100</t>
+          <t>01-000-2000</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="inlineStr">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>VOLLR01</t>
         </is>
       </c>
-      <c r="B29" s="2" t="inlineStr">
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>Vollrath Company</t>
         </is>
       </c>
-      <c r="C29" s="2" t="inlineStr">
+      <c r="C29" s="3" t="inlineStr">
         <is>
           <t>Commercial cooking equipment</t>
         </is>
       </c>
-      <c r="D29" s="2" t="inlineStr">
+      <c r="D29" s="3" t="inlineStr">
         <is>
           <t>1236 N 18th St</t>
         </is>
       </c>
-      <c r="E29" s="2" t="inlineStr"/>
-      <c r="F29" s="2" t="inlineStr"/>
-      <c r="G29" s="2" t="inlineStr">
+      <c r="E29" s="3" t="inlineStr"/>
+      <c r="F29" s="3" t="inlineStr"/>
+      <c r="G29" s="3" t="inlineStr">
         <is>
           <t>Sheboygan</t>
         </is>
       </c>
-      <c r="H29" s="2" t="inlineStr">
+      <c r="H29" s="3" t="inlineStr">
         <is>
           <t>WI</t>
         </is>
       </c>
-      <c r="I29" s="2" t="inlineStr">
+      <c r="I29" s="3" t="inlineStr">
         <is>
           <t>53081</t>
         </is>
       </c>
-      <c r="J29" s="2" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="K29" s="2" t="inlineStr">
-        <is>
-          <t>001-2100</t>
+      <c r="J29" s="3" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="K29" s="3" t="inlineStr">
+        <is>
+          <t>01-000-2000</t>
         </is>
       </c>
     </row>
@@ -1930,56 +1940,56 @@
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>001-2100</t>
+          <t>01-000-2000</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="inlineStr">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>WELBT01</t>
         </is>
       </c>
-      <c r="B31" s="2" t="inlineStr">
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>Welbilt Inc</t>
         </is>
       </c>
-      <c r="C31" s="2" t="inlineStr">
+      <c r="C31" s="3" t="inlineStr">
         <is>
           <t>Commercial foodservice equipment</t>
         </is>
       </c>
-      <c r="D31" s="2" t="inlineStr">
+      <c r="D31" s="3" t="inlineStr">
         <is>
           <t>2227 Welbilt Blvd</t>
         </is>
       </c>
-      <c r="E31" s="2" t="inlineStr"/>
-      <c r="F31" s="2" t="inlineStr"/>
-      <c r="G31" s="2" t="inlineStr">
+      <c r="E31" s="3" t="inlineStr"/>
+      <c r="F31" s="3" t="inlineStr"/>
+      <c r="G31" s="3" t="inlineStr">
         <is>
           <t>New Port Richey</t>
         </is>
       </c>
-      <c r="H31" s="2" t="inlineStr">
+      <c r="H31" s="3" t="inlineStr">
         <is>
           <t>FL</t>
         </is>
       </c>
-      <c r="I31" s="2" t="inlineStr">
+      <c r="I31" s="3" t="inlineStr">
         <is>
           <t>34655</t>
         </is>
       </c>
-      <c r="J31" s="2" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="K31" s="2" t="inlineStr">
-        <is>
-          <t>001-2100</t>
+      <c r="J31" s="3" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="K31" s="3" t="inlineStr">
+        <is>
+          <t>01-000-2000</t>
         </is>
       </c>
     </row>
@@ -2028,56 +2038,56 @@
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>001-2100</t>
+          <t>01-000-2000</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr">
+      <c r="A33" s="3" t="inlineStr">
         <is>
           <t>NCRCR01</t>
         </is>
       </c>
-      <c r="B33" s="2" t="inlineStr">
+      <c r="B33" s="3" t="inlineStr">
         <is>
           <t>NCR Corporation</t>
         </is>
       </c>
-      <c r="C33" s="2" t="inlineStr">
+      <c r="C33" s="3" t="inlineStr">
         <is>
           <t>POS systems and technology</t>
         </is>
       </c>
-      <c r="D33" s="2" t="inlineStr">
+      <c r="D33" s="3" t="inlineStr">
         <is>
           <t>864 Spring St NW</t>
         </is>
       </c>
-      <c r="E33" s="2" t="inlineStr"/>
-      <c r="F33" s="2" t="inlineStr"/>
-      <c r="G33" s="2" t="inlineStr">
+      <c r="E33" s="3" t="inlineStr"/>
+      <c r="F33" s="3" t="inlineStr"/>
+      <c r="G33" s="3" t="inlineStr">
         <is>
           <t>Atlanta</t>
         </is>
       </c>
-      <c r="H33" s="2" t="inlineStr">
+      <c r="H33" s="3" t="inlineStr">
         <is>
           <t>GA</t>
         </is>
       </c>
-      <c r="I33" s="2" t="inlineStr">
+      <c r="I33" s="3" t="inlineStr">
         <is>
           <t>30308</t>
         </is>
       </c>
-      <c r="J33" s="2" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="K33" s="2" t="inlineStr">
-        <is>
-          <t>001-2100</t>
+      <c r="J33" s="3" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="K33" s="3" t="inlineStr">
+        <is>
+          <t>01-000-2000</t>
         </is>
       </c>
     </row>
@@ -2130,56 +2140,56 @@
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>001-2100</t>
+          <t>01-000-2000</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="inlineStr">
+      <c r="A35" s="3" t="inlineStr">
         <is>
           <t>HRTLD01</t>
         </is>
       </c>
-      <c r="B35" s="2" t="inlineStr">
+      <c r="B35" s="3" t="inlineStr">
         <is>
           <t>Heartland Payment Systems</t>
         </is>
       </c>
-      <c r="C35" s="2" t="inlineStr">
+      <c r="C35" s="3" t="inlineStr">
         <is>
           <t>Payment processing services</t>
         </is>
       </c>
-      <c r="D35" s="2" t="inlineStr">
+      <c r="D35" s="3" t="inlineStr">
         <is>
           <t>90 Nassau St</t>
         </is>
       </c>
-      <c r="E35" s="2" t="inlineStr"/>
-      <c r="F35" s="2" t="inlineStr"/>
-      <c r="G35" s="2" t="inlineStr">
+      <c r="E35" s="3" t="inlineStr"/>
+      <c r="F35" s="3" t="inlineStr"/>
+      <c r="G35" s="3" t="inlineStr">
         <is>
           <t>Princeton</t>
         </is>
       </c>
-      <c r="H35" s="2" t="inlineStr">
+      <c r="H35" s="3" t="inlineStr">
         <is>
           <t>NJ</t>
         </is>
       </c>
-      <c r="I35" s="2" t="inlineStr">
+      <c r="I35" s="3" t="inlineStr">
         <is>
           <t>08542</t>
         </is>
       </c>
-      <c r="J35" s="2" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="K35" s="2" t="inlineStr">
-        <is>
-          <t>001-2100</t>
+      <c r="J35" s="3" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="K35" s="3" t="inlineStr">
+        <is>
+          <t>01-000-2000</t>
         </is>
       </c>
     </row>
@@ -2228,60 +2238,60 @@
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t>001-2100</t>
+          <t>01-000-2000</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="inlineStr">
+      <c r="A37" s="3" t="inlineStr">
         <is>
           <t>OPNTR01</t>
         </is>
       </c>
-      <c r="B37" s="2" t="inlineStr">
+      <c r="B37" s="3" t="inlineStr">
         <is>
           <t>OpenTable Inc</t>
         </is>
       </c>
-      <c r="C37" s="2" t="inlineStr">
+      <c r="C37" s="3" t="inlineStr">
         <is>
           <t>Reservation management platform</t>
         </is>
       </c>
-      <c r="D37" s="2" t="inlineStr">
+      <c r="D37" s="3" t="inlineStr">
         <is>
           <t>1 Montgomery St</t>
         </is>
       </c>
-      <c r="E37" s="2" t="inlineStr">
+      <c r="E37" s="3" t="inlineStr">
         <is>
           <t>Ste 700</t>
         </is>
       </c>
-      <c r="F37" s="2" t="inlineStr"/>
-      <c r="G37" s="2" t="inlineStr">
+      <c r="F37" s="3" t="inlineStr"/>
+      <c r="G37" s="3" t="inlineStr">
         <is>
           <t>San Francisco</t>
         </is>
       </c>
-      <c r="H37" s="2" t="inlineStr">
+      <c r="H37" s="3" t="inlineStr">
         <is>
           <t>CA</t>
         </is>
       </c>
-      <c r="I37" s="2" t="inlineStr">
+      <c r="I37" s="3" t="inlineStr">
         <is>
           <t>94104</t>
         </is>
       </c>
-      <c r="J37" s="2" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="K37" s="2" t="inlineStr">
-        <is>
-          <t>001-2100</t>
+      <c r="J37" s="3" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="K37" s="3" t="inlineStr">
+        <is>
+          <t>01-000-2000</t>
         </is>
       </c>
     </row>
@@ -2330,56 +2340,56 @@
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>001-2100</t>
+          <t>01-000-2000</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="inlineStr">
+      <c r="A39" s="3" t="inlineStr">
         <is>
           <t>RPSVC01</t>
         </is>
       </c>
-      <c r="B39" s="2" t="inlineStr">
+      <c r="B39" s="3" t="inlineStr">
         <is>
           <t>Republic Services</t>
         </is>
       </c>
-      <c r="C39" s="2" t="inlineStr">
+      <c r="C39" s="3" t="inlineStr">
         <is>
           <t>Waste management and recycling</t>
         </is>
       </c>
-      <c r="D39" s="2" t="inlineStr">
+      <c r="D39" s="3" t="inlineStr">
         <is>
           <t>18500 N Allied Way</t>
         </is>
       </c>
-      <c r="E39" s="2" t="inlineStr"/>
-      <c r="F39" s="2" t="inlineStr"/>
-      <c r="G39" s="2" t="inlineStr">
+      <c r="E39" s="3" t="inlineStr"/>
+      <c r="F39" s="3" t="inlineStr"/>
+      <c r="G39" s="3" t="inlineStr">
         <is>
           <t>Phoenix</t>
         </is>
       </c>
-      <c r="H39" s="2" t="inlineStr">
+      <c r="H39" s="3" t="inlineStr">
         <is>
           <t>AZ</t>
         </is>
       </c>
-      <c r="I39" s="2" t="inlineStr">
+      <c r="I39" s="3" t="inlineStr">
         <is>
           <t>85054</t>
         </is>
       </c>
-      <c r="J39" s="2" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="K39" s="2" t="inlineStr">
-        <is>
-          <t>001-2100</t>
+      <c r="J39" s="3" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="K39" s="3" t="inlineStr">
+        <is>
+          <t>01-000-2000</t>
         </is>
       </c>
     </row>
@@ -2428,56 +2438,56 @@
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>001-2100</t>
+          <t>01-000-2000</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="inlineStr">
+      <c r="A41" s="3" t="inlineStr">
         <is>
           <t>HRTFD01</t>
         </is>
       </c>
-      <c r="B41" s="2" t="inlineStr">
+      <c r="B41" s="3" t="inlineStr">
         <is>
           <t>Hartford Financial Services</t>
         </is>
       </c>
-      <c r="C41" s="2" t="inlineStr">
+      <c r="C41" s="3" t="inlineStr">
         <is>
           <t>Commercial insurance</t>
         </is>
       </c>
-      <c r="D41" s="2" t="inlineStr">
+      <c r="D41" s="3" t="inlineStr">
         <is>
           <t>1 Hartford Plz</t>
         </is>
       </c>
-      <c r="E41" s="2" t="inlineStr"/>
-      <c r="F41" s="2" t="inlineStr"/>
-      <c r="G41" s="2" t="inlineStr">
+      <c r="E41" s="3" t="inlineStr"/>
+      <c r="F41" s="3" t="inlineStr"/>
+      <c r="G41" s="3" t="inlineStr">
         <is>
           <t>Hartford</t>
         </is>
       </c>
-      <c r="H41" s="2" t="inlineStr">
+      <c r="H41" s="3" t="inlineStr">
         <is>
           <t>CT</t>
         </is>
       </c>
-      <c r="I41" s="2" t="inlineStr">
+      <c r="I41" s="3" t="inlineStr">
         <is>
           <t>06155</t>
         </is>
       </c>
-      <c r="J41" s="2" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="K41" s="2" t="inlineStr">
-        <is>
-          <t>001-2100</t>
+      <c r="J41" s="3" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="K41" s="3" t="inlineStr">
+        <is>
+          <t>01-000-2000</t>
         </is>
       </c>
     </row>
@@ -2530,56 +2540,56 @@
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>001-2100</t>
+          <t>01-000-2000</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="inlineStr">
+      <c r="A43" s="3" t="inlineStr">
         <is>
           <t>SPLXG01</t>
         </is>
       </c>
-      <c r="B43" s="2" t="inlineStr">
+      <c r="B43" s="3" t="inlineStr">
         <is>
           <t>Simplex-Grinnell</t>
         </is>
       </c>
-      <c r="C43" s="2" t="inlineStr">
+      <c r="C43" s="3" t="inlineStr">
         <is>
           <t>Fire suppression and safety</t>
         </is>
       </c>
-      <c r="D43" s="2" t="inlineStr">
+      <c r="D43" s="3" t="inlineStr">
         <is>
           <t>50 Technology Dr</t>
         </is>
       </c>
-      <c r="E43" s="2" t="inlineStr"/>
-      <c r="F43" s="2" t="inlineStr"/>
-      <c r="G43" s="2" t="inlineStr">
+      <c r="E43" s="3" t="inlineStr"/>
+      <c r="F43" s="3" t="inlineStr"/>
+      <c r="G43" s="3" t="inlineStr">
         <is>
           <t>Westminster</t>
         </is>
       </c>
-      <c r="H43" s="2" t="inlineStr">
+      <c r="H43" s="3" t="inlineStr">
         <is>
           <t>MA</t>
         </is>
       </c>
-      <c r="I43" s="2" t="inlineStr">
+      <c r="I43" s="3" t="inlineStr">
         <is>
           <t>01441</t>
         </is>
       </c>
-      <c r="J43" s="2" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="K43" s="2" t="inlineStr">
-        <is>
-          <t>001-2100</t>
+      <c r="J43" s="3" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="K43" s="3" t="inlineStr">
+        <is>
+          <t>01-000-2000</t>
         </is>
       </c>
     </row>
@@ -2628,56 +2638,56 @@
       </c>
       <c r="K44" s="2" t="inlineStr">
         <is>
-          <t>001-2100</t>
+          <t>01-000-2000</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="inlineStr">
+      <c r="A45" s="3" t="inlineStr">
         <is>
           <t>ZAYOG01</t>
         </is>
       </c>
-      <c r="B45" s="2" t="inlineStr">
+      <c r="B45" s="3" t="inlineStr">
         <is>
           <t>Zayo Group</t>
         </is>
       </c>
-      <c r="C45" s="2" t="inlineStr">
+      <c r="C45" s="3" t="inlineStr">
         <is>
           <t>Fiber internet and connectivity</t>
         </is>
       </c>
-      <c r="D45" s="2" t="inlineStr">
+      <c r="D45" s="3" t="inlineStr">
         <is>
           <t>1821 30th St</t>
         </is>
       </c>
-      <c r="E45" s="2" t="inlineStr"/>
-      <c r="F45" s="2" t="inlineStr"/>
-      <c r="G45" s="2" t="inlineStr">
+      <c r="E45" s="3" t="inlineStr"/>
+      <c r="F45" s="3" t="inlineStr"/>
+      <c r="G45" s="3" t="inlineStr">
         <is>
           <t>Boulder</t>
         </is>
       </c>
-      <c r="H45" s="2" t="inlineStr">
+      <c r="H45" s="3" t="inlineStr">
         <is>
           <t>CO</t>
         </is>
       </c>
-      <c r="I45" s="2" t="inlineStr">
+      <c r="I45" s="3" t="inlineStr">
         <is>
           <t>80301</t>
         </is>
       </c>
-      <c r="J45" s="2" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="K45" s="2" t="inlineStr">
-        <is>
-          <t>001-2100</t>
+      <c r="J45" s="3" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="K45" s="3" t="inlineStr">
+        <is>
+          <t>01-000-2000</t>
         </is>
       </c>
     </row>
@@ -2726,56 +2736,56 @@
       </c>
       <c r="K46" s="2" t="inlineStr">
         <is>
-          <t>001-2100</t>
+          <t>01-000-2000</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="inlineStr">
+      <c r="A47" s="3" t="inlineStr">
         <is>
           <t>ONCOR01</t>
         </is>
       </c>
-      <c r="B47" s="2" t="inlineStr">
+      <c r="B47" s="3" t="inlineStr">
         <is>
           <t>Oncor Electric Delivery</t>
         </is>
       </c>
-      <c r="C47" s="2" t="inlineStr">
+      <c r="C47" s="3" t="inlineStr">
         <is>
           <t>Electric utility services</t>
         </is>
       </c>
-      <c r="D47" s="2" t="inlineStr">
+      <c r="D47" s="3" t="inlineStr">
         <is>
           <t>1616 Woodall Rodgers Fwy</t>
         </is>
       </c>
-      <c r="E47" s="2" t="inlineStr"/>
-      <c r="F47" s="2" t="inlineStr"/>
-      <c r="G47" s="2" t="inlineStr">
+      <c r="E47" s="3" t="inlineStr"/>
+      <c r="F47" s="3" t="inlineStr"/>
+      <c r="G47" s="3" t="inlineStr">
         <is>
           <t>Dallas</t>
         </is>
       </c>
-      <c r="H47" s="2" t="inlineStr">
+      <c r="H47" s="3" t="inlineStr">
         <is>
           <t>TX</t>
         </is>
       </c>
-      <c r="I47" s="2" t="inlineStr">
+      <c r="I47" s="3" t="inlineStr">
         <is>
           <t>75202</t>
         </is>
       </c>
-      <c r="J47" s="2" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="K47" s="2" t="inlineStr">
-        <is>
-          <t>001-2100</t>
+      <c r="J47" s="3" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="K47" s="3" t="inlineStr">
+        <is>
+          <t>01-000-2000</t>
         </is>
       </c>
     </row>
@@ -2828,56 +2838,56 @@
       </c>
       <c r="K48" s="2" t="inlineStr">
         <is>
-          <t>001-2100</t>
+          <t>01-000-2000</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="inlineStr">
+      <c r="A49" s="3" t="inlineStr">
         <is>
           <t>SEALE01</t>
         </is>
       </c>
-      <c r="B49" s="2" t="inlineStr">
+      <c r="B49" s="3" t="inlineStr">
         <is>
           <t>Sealand Food</t>
         </is>
       </c>
-      <c r="C49" s="2" t="inlineStr">
+      <c r="C49" s="3" t="inlineStr">
         <is>
           <t>Specialty seafood distributor</t>
         </is>
       </c>
-      <c r="D49" s="2" t="inlineStr">
+      <c r="D49" s="3" t="inlineStr">
         <is>
           <t>3420 Ocean Dr</t>
         </is>
       </c>
-      <c r="E49" s="2" t="inlineStr"/>
-      <c r="F49" s="2" t="inlineStr"/>
-      <c r="G49" s="2" t="inlineStr">
+      <c r="E49" s="3" t="inlineStr"/>
+      <c r="F49" s="3" t="inlineStr"/>
+      <c r="G49" s="3" t="inlineStr">
         <is>
           <t>Virginia Beach</t>
         </is>
       </c>
-      <c r="H49" s="2" t="inlineStr">
+      <c r="H49" s="3" t="inlineStr">
         <is>
           <t>VA</t>
         </is>
       </c>
-      <c r="I49" s="2" t="inlineStr">
+      <c r="I49" s="3" t="inlineStr">
         <is>
           <t>23451</t>
         </is>
       </c>
-      <c r="J49" s="2" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="K49" s="2" t="inlineStr">
-        <is>
-          <t>001-2100</t>
+      <c r="J49" s="3" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="K49" s="3" t="inlineStr">
+        <is>
+          <t>01-000-2000</t>
         </is>
       </c>
     </row>
@@ -2930,56 +2940,56 @@
       </c>
       <c r="K50" s="2" t="inlineStr">
         <is>
-          <t>001-2100</t>
+          <t>01-000-2000</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="2" t="inlineStr">
+      <c r="A51" s="3" t="inlineStr">
         <is>
           <t>CHURF01</t>
         </is>
       </c>
-      <c r="B51" s="2" t="inlineStr">
+      <c r="B51" s="3" t="inlineStr">
         <is>
           <t>Chur Farms Produce</t>
         </is>
       </c>
-      <c r="C51" s="2" t="inlineStr">
+      <c r="C51" s="3" t="inlineStr">
         <is>
           <t>Local fresh produce supplier</t>
         </is>
       </c>
-      <c r="D51" s="2" t="inlineStr">
+      <c r="D51" s="3" t="inlineStr">
         <is>
           <t>4500 Farm Rd 55</t>
         </is>
       </c>
-      <c r="E51" s="2" t="inlineStr"/>
-      <c r="F51" s="2" t="inlineStr"/>
-      <c r="G51" s="2" t="inlineStr">
+      <c r="E51" s="3" t="inlineStr"/>
+      <c r="F51" s="3" t="inlineStr"/>
+      <c r="G51" s="3" t="inlineStr">
         <is>
           <t>Hereford</t>
         </is>
       </c>
-      <c r="H51" s="2" t="inlineStr">
+      <c r="H51" s="3" t="inlineStr">
         <is>
           <t>TX</t>
         </is>
       </c>
-      <c r="I51" s="2" t="inlineStr">
+      <c r="I51" s="3" t="inlineStr">
         <is>
           <t>79045</t>
         </is>
       </c>
-      <c r="J51" s="2" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="K51" s="2" t="inlineStr">
-        <is>
-          <t>001-2100</t>
+      <c r="J51" s="3" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="K51" s="3" t="inlineStr">
+        <is>
+          <t>01-000-2000</t>
         </is>
       </c>
     </row>

</xml_diff>